<commit_message>
Add hero-tabs block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (9):
- blocks/hero-tabs/hero-tabs.css
- blocks/hero-tabs/hero-tabs.js
- tools/importer/import-products.bundle.js
- tools/importer/import-products.js
- tools/importer/parsers/hero-tabs.js
- tools/importer/reports/en/products.report.json
- tools/importer/reports/en/products/7up.report.json
- tools/importer/reports/import-products-7up.report.xlsx
- tools/importer/reports/import-products.report.xlsx
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-products-7up.report.xlsx
+++ b/tools/importer/reports/import-products-7up.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="147">
   <si>
     <t>_reportFile</t>
   </si>
@@ -64,7 +64,7 @@
     <t>en/products.report.json</t>
   </si>
   <si>
-    <t>["carousel-product","cards-nutrition","cards-nutrition","cards-nutrition","cards-nutrition","cards-nutrition","cards-nutrition"]</t>
+    <t>["hero-tabs"]</t>
   </si>
   <si>
     <t>en/products</t>
@@ -73,7 +73,7 @@
     <t>products</t>
   </si>
   <si>
-    <t>2026-09-10T18:31:45.028Z</t>
+    <t>2026-09-14T17:55:54.351Z</t>
   </si>
   <si>
     <t>https://www.7up.com/en/products</t>
@@ -103,16 +103,13 @@
     <t>en/products/7up.report.json</t>
   </si>
   <si>
-    <t>["hero-tabs"]</t>
-  </si>
-  <si>
     <t>en/products/7up</t>
   </si>
   <si>
     <t>products-7up</t>
   </si>
   <si>
-    <t>2026-09-14T17:28:52.031Z</t>
+    <t>2026-09-14T17:57:19.774Z</t>
   </si>
   <si>
     <t/>
@@ -846,7 +843,8 @@
   <dimension ref="A1:H27"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="2" width="50" customWidth="1"/>
+    <col min="1" max="1" width="50" customWidth="1"/>
+    <col min="2" max="2" width="45" customWidth="1"/>
     <col min="3" max="3" width="38" customWidth="1"/>
     <col min="5" max="5" width="15" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
@@ -963,597 +961,597 @@
         <v>29</v>
       </c>
       <c r="B5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" t="s">
         <v>30</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
         <v>31</v>
       </c>
-      <c r="D5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>32</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>33</v>
       </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>34</v>
-      </c>
-      <c r="H5" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" t="s">
         <v>37</v>
       </c>
-      <c r="C6" t="s">
-        <v>38</v>
-      </c>
       <c r="D6" t="s">
         <v>11</v>
       </c>
       <c r="E6" t="s">
+        <v>38</v>
+      </c>
+      <c r="F6" t="s">
         <v>39</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>40</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>41</v>
-      </c>
-      <c r="H6" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" t="s">
         <v>43</v>
       </c>
-      <c r="B7" t="s">
-        <v>37</v>
-      </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" t="s">
+        <v>38</v>
+      </c>
+      <c r="F7" t="s">
         <v>44</v>
       </c>
-      <c r="D7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E7" t="s">
-        <v>39</v>
-      </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>45</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" t="s">
         <v>46</v>
-      </c>
-      <c r="H7" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>47</v>
+      </c>
+      <c r="B8" t="s">
+        <v>36</v>
+      </c>
+      <c r="C8" t="s">
         <v>48</v>
       </c>
-      <c r="B8" t="s">
-        <v>37</v>
-      </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F8" t="s">
         <v>49</v>
       </c>
-      <c r="D8" t="s">
-        <v>11</v>
-      </c>
-      <c r="E8" t="s">
-        <v>39</v>
-      </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>50</v>
       </c>
-      <c r="G8" t="s">
+      <c r="H8" t="s">
         <v>51</v>
-      </c>
-      <c r="H8" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>52</v>
+      </c>
+      <c r="B9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" t="s">
         <v>53</v>
       </c>
-      <c r="B9" t="s">
-        <v>37</v>
-      </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" t="s">
+        <v>38</v>
+      </c>
+      <c r="F9" t="s">
         <v>54</v>
       </c>
-      <c r="D9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E9" t="s">
-        <v>39</v>
-      </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>55</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
         <v>56</v>
-      </c>
-      <c r="H9" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>57</v>
+      </c>
+      <c r="B10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" t="s">
         <v>58</v>
       </c>
-      <c r="B10" t="s">
-        <v>37</v>
-      </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" t="s">
+        <v>38</v>
+      </c>
+      <c r="F10" t="s">
         <v>59</v>
       </c>
-      <c r="D10" t="s">
-        <v>11</v>
-      </c>
-      <c r="E10" t="s">
-        <v>39</v>
-      </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>60</v>
       </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>61</v>
-      </c>
-      <c r="H10" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>62</v>
+      </c>
+      <c r="B11" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" t="s">
         <v>63</v>
       </c>
-      <c r="B11" t="s">
-        <v>37</v>
-      </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" t="s">
+        <v>38</v>
+      </c>
+      <c r="F11" t="s">
         <v>64</v>
       </c>
-      <c r="D11" t="s">
-        <v>11</v>
-      </c>
-      <c r="E11" t="s">
-        <v>39</v>
-      </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>65</v>
       </c>
-      <c r="G11" t="s">
+      <c r="H11" t="s">
         <v>66</v>
-      </c>
-      <c r="H11" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>67</v>
+      </c>
+      <c r="B12" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" t="s">
         <v>68</v>
       </c>
-      <c r="B12" t="s">
-        <v>37</v>
-      </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" t="s">
+        <v>38</v>
+      </c>
+      <c r="F12" t="s">
         <v>69</v>
       </c>
-      <c r="D12" t="s">
-        <v>11</v>
-      </c>
-      <c r="E12" t="s">
-        <v>39</v>
-      </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
         <v>70</v>
       </c>
-      <c r="G12" t="s">
+      <c r="H12" t="s">
         <v>71</v>
-      </c>
-      <c r="H12" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>72</v>
+      </c>
+      <c r="B13" t="s">
+        <v>36</v>
+      </c>
+      <c r="C13" t="s">
         <v>73</v>
       </c>
-      <c r="B13" t="s">
-        <v>37</v>
-      </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" t="s">
+        <v>38</v>
+      </c>
+      <c r="F13" t="s">
         <v>74</v>
       </c>
-      <c r="D13" t="s">
-        <v>11</v>
-      </c>
-      <c r="E13" t="s">
-        <v>39</v>
-      </c>
-      <c r="F13" t="s">
+      <c r="G13" t="s">
         <v>75</v>
       </c>
-      <c r="G13" t="s">
+      <c r="H13" t="s">
         <v>76</v>
-      </c>
-      <c r="H13" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>77</v>
+      </c>
+      <c r="B14" t="s">
+        <v>36</v>
+      </c>
+      <c r="C14" t="s">
         <v>78</v>
       </c>
-      <c r="B14" t="s">
-        <v>37</v>
-      </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" t="s">
+        <v>38</v>
+      </c>
+      <c r="F14" t="s">
         <v>79</v>
       </c>
-      <c r="D14" t="s">
-        <v>11</v>
-      </c>
-      <c r="E14" t="s">
-        <v>39</v>
-      </c>
-      <c r="F14" t="s">
+      <c r="G14" t="s">
         <v>80</v>
       </c>
-      <c r="G14" t="s">
+      <c r="H14" t="s">
         <v>81</v>
-      </c>
-      <c r="H14" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>82</v>
+      </c>
+      <c r="B15" t="s">
+        <v>36</v>
+      </c>
+      <c r="C15" t="s">
         <v>83</v>
       </c>
-      <c r="B15" t="s">
-        <v>37</v>
-      </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" t="s">
+        <v>38</v>
+      </c>
+      <c r="F15" t="s">
         <v>84</v>
       </c>
-      <c r="D15" t="s">
-        <v>11</v>
-      </c>
-      <c r="E15" t="s">
-        <v>39</v>
-      </c>
-      <c r="F15" t="s">
+      <c r="G15" t="s">
         <v>85</v>
       </c>
-      <c r="G15" t="s">
+      <c r="H15" t="s">
         <v>86</v>
-      </c>
-      <c r="H15" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>87</v>
+      </c>
+      <c r="B16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C16" t="s">
         <v>88</v>
       </c>
-      <c r="B16" t="s">
-        <v>37</v>
-      </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
+        <v>11</v>
+      </c>
+      <c r="E16" t="s">
+        <v>38</v>
+      </c>
+      <c r="F16" t="s">
         <v>89</v>
       </c>
-      <c r="D16" t="s">
-        <v>11</v>
-      </c>
-      <c r="E16" t="s">
-        <v>39</v>
-      </c>
-      <c r="F16" t="s">
+      <c r="G16" t="s">
         <v>90</v>
       </c>
-      <c r="G16" t="s">
+      <c r="H16" t="s">
         <v>91</v>
-      </c>
-      <c r="H16" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>92</v>
+      </c>
+      <c r="B17" t="s">
+        <v>36</v>
+      </c>
+      <c r="C17" t="s">
         <v>93</v>
       </c>
-      <c r="B17" t="s">
-        <v>37</v>
-      </c>
-      <c r="C17" t="s">
+      <c r="D17" t="s">
+        <v>11</v>
+      </c>
+      <c r="E17" t="s">
+        <v>38</v>
+      </c>
+      <c r="F17" t="s">
         <v>94</v>
       </c>
-      <c r="D17" t="s">
-        <v>11</v>
-      </c>
-      <c r="E17" t="s">
-        <v>39</v>
-      </c>
-      <c r="F17" t="s">
+      <c r="G17" t="s">
         <v>95</v>
       </c>
-      <c r="G17" t="s">
+      <c r="H17" t="s">
         <v>96</v>
-      </c>
-      <c r="H17" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>97</v>
+      </c>
+      <c r="B18" t="s">
+        <v>36</v>
+      </c>
+      <c r="C18" t="s">
         <v>98</v>
       </c>
-      <c r="B18" t="s">
-        <v>37</v>
-      </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
+        <v>11</v>
+      </c>
+      <c r="E18" t="s">
+        <v>38</v>
+      </c>
+      <c r="F18" t="s">
         <v>99</v>
       </c>
-      <c r="D18" t="s">
-        <v>11</v>
-      </c>
-      <c r="E18" t="s">
-        <v>39</v>
-      </c>
-      <c r="F18" t="s">
+      <c r="G18" t="s">
         <v>100</v>
       </c>
-      <c r="G18" t="s">
+      <c r="H18" t="s">
         <v>101</v>
-      </c>
-      <c r="H18" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>102</v>
+      </c>
+      <c r="B19" t="s">
+        <v>36</v>
+      </c>
+      <c r="C19" t="s">
         <v>103</v>
       </c>
-      <c r="B19" t="s">
-        <v>37</v>
-      </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
+        <v>11</v>
+      </c>
+      <c r="E19" t="s">
+        <v>38</v>
+      </c>
+      <c r="F19" t="s">
         <v>104</v>
       </c>
-      <c r="D19" t="s">
-        <v>11</v>
-      </c>
-      <c r="E19" t="s">
-        <v>39</v>
-      </c>
-      <c r="F19" t="s">
+      <c r="G19" t="s">
         <v>105</v>
       </c>
-      <c r="G19" t="s">
+      <c r="H19" t="s">
         <v>106</v>
-      </c>
-      <c r="H19" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>107</v>
+      </c>
+      <c r="B20" t="s">
+        <v>36</v>
+      </c>
+      <c r="C20" t="s">
         <v>108</v>
       </c>
-      <c r="B20" t="s">
-        <v>37</v>
-      </c>
-      <c r="C20" t="s">
+      <c r="D20" t="s">
+        <v>11</v>
+      </c>
+      <c r="E20" t="s">
+        <v>38</v>
+      </c>
+      <c r="F20" t="s">
         <v>109</v>
       </c>
-      <c r="D20" t="s">
-        <v>11</v>
-      </c>
-      <c r="E20" t="s">
-        <v>39</v>
-      </c>
-      <c r="F20" t="s">
+      <c r="G20" t="s">
         <v>110</v>
       </c>
-      <c r="G20" t="s">
+      <c r="H20" t="s">
         <v>111</v>
-      </c>
-      <c r="H20" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>112</v>
+      </c>
+      <c r="B21" t="s">
+        <v>36</v>
+      </c>
+      <c r="C21" t="s">
         <v>113</v>
       </c>
-      <c r="B21" t="s">
-        <v>37</v>
-      </c>
-      <c r="C21" t="s">
+      <c r="D21" t="s">
+        <v>11</v>
+      </c>
+      <c r="E21" t="s">
+        <v>38</v>
+      </c>
+      <c r="F21" t="s">
         <v>114</v>
       </c>
-      <c r="D21" t="s">
-        <v>11</v>
-      </c>
-      <c r="E21" t="s">
-        <v>39</v>
-      </c>
-      <c r="F21" t="s">
+      <c r="G21" t="s">
         <v>115</v>
       </c>
-      <c r="G21" t="s">
+      <c r="H21" t="s">
         <v>116</v>
-      </c>
-      <c r="H21" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>117</v>
+      </c>
+      <c r="B22" t="s">
+        <v>36</v>
+      </c>
+      <c r="C22" t="s">
         <v>118</v>
       </c>
-      <c r="B22" t="s">
-        <v>37</v>
-      </c>
-      <c r="C22" t="s">
+      <c r="D22" t="s">
+        <v>11</v>
+      </c>
+      <c r="E22" t="s">
+        <v>38</v>
+      </c>
+      <c r="F22" t="s">
         <v>119</v>
       </c>
-      <c r="D22" t="s">
-        <v>11</v>
-      </c>
-      <c r="E22" t="s">
-        <v>39</v>
-      </c>
-      <c r="F22" t="s">
+      <c r="G22" t="s">
         <v>120</v>
       </c>
-      <c r="G22" t="s">
+      <c r="H22" t="s">
         <v>121</v>
-      </c>
-      <c r="H22" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>122</v>
+      </c>
+      <c r="B23" t="s">
+        <v>36</v>
+      </c>
+      <c r="C23" t="s">
         <v>123</v>
       </c>
-      <c r="B23" t="s">
-        <v>37</v>
-      </c>
-      <c r="C23" t="s">
+      <c r="D23" t="s">
+        <v>11</v>
+      </c>
+      <c r="E23" t="s">
+        <v>38</v>
+      </c>
+      <c r="F23" t="s">
         <v>124</v>
       </c>
-      <c r="D23" t="s">
-        <v>11</v>
-      </c>
-      <c r="E23" t="s">
-        <v>39</v>
-      </c>
-      <c r="F23" t="s">
+      <c r="G23" t="s">
         <v>125</v>
       </c>
-      <c r="G23" t="s">
+      <c r="H23" t="s">
         <v>126</v>
-      </c>
-      <c r="H23" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>127</v>
+      </c>
+      <c r="B24" t="s">
+        <v>36</v>
+      </c>
+      <c r="C24" t="s">
         <v>128</v>
       </c>
-      <c r="B24" t="s">
-        <v>37</v>
-      </c>
-      <c r="C24" t="s">
+      <c r="D24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E24" t="s">
+        <v>38</v>
+      </c>
+      <c r="F24" t="s">
         <v>129</v>
       </c>
-      <c r="D24" t="s">
-        <v>11</v>
-      </c>
-      <c r="E24" t="s">
-        <v>39</v>
-      </c>
-      <c r="F24" t="s">
+      <c r="G24" t="s">
         <v>130</v>
       </c>
-      <c r="G24" t="s">
+      <c r="H24" t="s">
         <v>131</v>
-      </c>
-      <c r="H24" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>132</v>
+      </c>
+      <c r="B25" t="s">
+        <v>36</v>
+      </c>
+      <c r="C25" t="s">
         <v>133</v>
       </c>
-      <c r="B25" t="s">
-        <v>37</v>
-      </c>
-      <c r="C25" t="s">
+      <c r="D25" t="s">
+        <v>11</v>
+      </c>
+      <c r="E25" t="s">
+        <v>38</v>
+      </c>
+      <c r="F25" t="s">
         <v>134</v>
       </c>
-      <c r="D25" t="s">
-        <v>11</v>
-      </c>
-      <c r="E25" t="s">
-        <v>39</v>
-      </c>
-      <c r="F25" t="s">
+      <c r="G25" t="s">
         <v>135</v>
       </c>
-      <c r="G25" t="s">
+      <c r="H25" t="s">
         <v>136</v>
-      </c>
-      <c r="H25" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>137</v>
+      </c>
+      <c r="B26" t="s">
+        <v>36</v>
+      </c>
+      <c r="C26" t="s">
         <v>138</v>
       </c>
-      <c r="B26" t="s">
-        <v>37</v>
-      </c>
-      <c r="C26" t="s">
+      <c r="D26" t="s">
+        <v>11</v>
+      </c>
+      <c r="E26" t="s">
+        <v>38</v>
+      </c>
+      <c r="F26" t="s">
         <v>139</v>
       </c>
-      <c r="D26" t="s">
-        <v>11</v>
-      </c>
-      <c r="E26" t="s">
-        <v>39</v>
-      </c>
-      <c r="F26" t="s">
+      <c r="G26" t="s">
         <v>140</v>
       </c>
-      <c r="G26" t="s">
+      <c r="H26" t="s">
         <v>141</v>
-      </c>
-      <c r="H26" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>142</v>
+      </c>
+      <c r="B27" t="s">
+        <v>36</v>
+      </c>
+      <c r="C27" t="s">
         <v>143</v>
       </c>
-      <c r="B27" t="s">
-        <v>37</v>
-      </c>
-      <c r="C27" t="s">
+      <c r="D27" t="s">
+        <v>11</v>
+      </c>
+      <c r="E27" t="s">
+        <v>38</v>
+      </c>
+      <c r="F27" t="s">
         <v>144</v>
       </c>
-      <c r="D27" t="s">
-        <v>11</v>
-      </c>
-      <c r="E27" t="s">
-        <v>39</v>
-      </c>
-      <c r="F27" t="s">
+      <c r="G27" t="s">
         <v>145</v>
       </c>
-      <c r="G27" t="s">
+      <c r="H27" t="s">
         <v>146</v>
-      </c>
-      <c r="H27" t="s">
-        <v>147</v>
       </c>
     </row>
   </sheetData>

</xml_diff>